<commit_message>
Update Excel data with latest package assignments
Synced from source file - 2YM now correctly assigned to
"Payments - basic" package. No unassigned items remain.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/data/treasury-scope-items.xlsx
+++ b/docs/data/treasury-scope-items.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JanRuman\Downloads\Public Cloud\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BEA32F3-6781-41BB-AE13-5012C3B671B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7572824D-6792-4B9B-AA78-8A79D9D3CF86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11835" uniqueCount="1746">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11836" uniqueCount="1746">
   <si>
     <t>Erweiterte Bankkontenverwaltung (J77)</t>
   </si>
@@ -5966,7 +5966,9 @@
         <v>627</v>
       </c>
       <c r="J5" s="2"/>
-      <c r="K5" s="2"/>
+      <c r="K5" s="8" t="s">
+        <v>1724</v>
+      </c>
       <c r="L5" s="2">
         <v>2</v>
       </c>
@@ -6109,9 +6111,8 @@
       <c r="K9" s="2" t="s">
         <v>1744</v>
       </c>
-      <c r="L9" s="2" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
+      <c r="L9" s="2">
+        <v>5</v>
       </c>
       <c r="M9" t="s">
         <v>706</v>
@@ -6250,9 +6251,8 @@
       <c r="K13" s="2" t="s">
         <v>1734</v>
       </c>
-      <c r="L13" s="2" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
+      <c r="L13" s="2">
+        <v>5</v>
       </c>
       <c r="M13" t="s">
         <v>719</v>
@@ -6517,9 +6517,8 @@
       <c r="K21" s="2" t="s">
         <v>1735</v>
       </c>
-      <c r="L21" s="2" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
+      <c r="L21" s="2">
+        <v>6</v>
       </c>
       <c r="M21" t="s">
         <v>738</v>

</xml_diff>